<commit_message>
description and excel sheet modifications
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/pvest/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C169DEFC-9BC8-F246-B9AA-8573295CB489}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159EDE11-BF95-5D49-BFF6-A4914956087A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="578" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="procedure" sheetId="18" r:id="rId1"/>
@@ -21009,7 +21009,7 @@
         <v>3.7215533488415815</v>
       </c>
       <c r="H8" s="6">
-        <f>(E8-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" ref="H8:H14" si="3">(E8-N$10/100)/(1-N$10/100)</f>
         <v>0.95687545977321131</v>
       </c>
       <c r="I8" s="9">
@@ -21021,11 +21021,11 @@
         <v>4.3124540226788639</v>
       </c>
       <c r="K8" s="10">
-        <f>-1/($K$29+$K$28*G8)</f>
+        <f t="shared" ref="K8:K14" si="4">-1/($K$29+$K$28*G8)</f>
         <v>-2.5649159437272537</v>
       </c>
       <c r="L8" s="10">
-        <f>A8-K8</f>
+        <f t="shared" ref="L8:L14" si="5">A8-K8</f>
         <v>2.0429159437272535</v>
       </c>
       <c r="M8" s="62" t="s">
@@ -21052,39 +21052,39 @@
         <v>1.5744499999999999</v>
       </c>
       <c r="D9" s="7">
-        <f t="shared" ref="D9" si="3">C9-$B$3-$B$4</f>
+        <f t="shared" ref="D9" si="6">C9-$B$3-$B$4</f>
         <v>0.12533</v>
       </c>
       <c r="E9" s="6">
-        <f t="shared" ref="E9" si="4">(D9/$B$29)</f>
+        <f t="shared" ref="E9" si="7">(D9/$B$29)</f>
         <v>0.89547886595841819</v>
       </c>
       <c r="F9" s="9">
-        <f t="shared" ref="F9" si="5">100*E9</f>
+        <f t="shared" ref="F9" si="8">100*E9</f>
         <v>89.547886595841817</v>
       </c>
       <c r="G9" s="9">
-        <f t="shared" ref="G9" si="6">100-F9</f>
+        <f t="shared" ref="G9" si="9">100-F9</f>
         <v>10.452113404158183</v>
       </c>
       <c r="H9" s="6">
-        <f>(E9-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" si="3"/>
         <v>0.87888321281411175</v>
       </c>
       <c r="I9" s="9">
-        <f t="shared" ref="I9" si="7">H9*100</f>
+        <f t="shared" ref="I9" si="10">H9*100</f>
         <v>87.88832128141118</v>
       </c>
       <c r="J9" s="9">
-        <f t="shared" ref="J9:J14" si="8">100-I9</f>
+        <f t="shared" ref="J9:J14" si="11">100-I9</f>
         <v>12.11167871858882</v>
       </c>
       <c r="K9" s="10">
-        <f>-1/($K$29+$K$28*G9)</f>
+        <f t="shared" si="4"/>
         <v>-2.7925270242392881</v>
       </c>
       <c r="L9" s="10">
-        <f>A9-K9</f>
+        <f t="shared" si="5"/>
         <v>1.4975270242392882</v>
       </c>
       <c r="M9" s="67" t="s">
@@ -21111,39 +21111,39 @@
         <v>1.56304</v>
       </c>
       <c r="D10" s="26">
-        <f t="shared" ref="D10:D20" si="9">C10-$B$3-$B$4</f>
+        <f t="shared" ref="D10:D20" si="12">C10-$B$3-$B$4</f>
         <v>0.11392000000000008</v>
       </c>
       <c r="E10" s="27">
-        <f t="shared" ref="E10:E20" si="10">(D10/$B$29)</f>
+        <f t="shared" ref="E10:E20" si="13">(D10/$B$29)</f>
         <v>0.81395477866419108</v>
       </c>
       <c r="F10" s="28">
-        <f t="shared" ref="F10:F20" si="11">100*E10</f>
+        <f t="shared" ref="F10:F20" si="14">100*E10</f>
         <v>81.395477866419114</v>
       </c>
       <c r="G10" s="28">
-        <f t="shared" ref="G10:G20" si="12">100-F10</f>
+        <f t="shared" ref="G10:G20" si="15">100-F10</f>
         <v>18.604522133580886</v>
       </c>
       <c r="H10" s="27">
-        <f>(E10-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" si="3"/>
         <v>0.78441489669910935</v>
       </c>
       <c r="I10" s="28">
-        <f t="shared" ref="I10:I20" si="13">H10*100</f>
+        <f t="shared" ref="I10:I20" si="16">H10*100</f>
         <v>78.441489669910936</v>
       </c>
       <c r="J10" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>21.558510330089064</v>
       </c>
       <c r="K10" s="29">
-        <f>-1/($K$29+$K$28*G10)</f>
+        <f t="shared" si="4"/>
         <v>-3.1288354329597761</v>
       </c>
       <c r="L10" s="29">
-        <f>A10-K10</f>
+        <f t="shared" si="5"/>
         <v>0.72383543295977626</v>
       </c>
       <c r="M10" s="62" t="s">
@@ -21170,39 +21170,39 @@
         <v>1.5527899999999999</v>
       </c>
       <c r="D11" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.10366999999999998</v>
       </c>
       <c r="E11" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.74071885449540575</v>
       </c>
       <c r="F11" s="9">
+        <f t="shared" si="14"/>
+        <v>74.071885449540574</v>
+      </c>
+      <c r="G11" s="9">
+        <f t="shared" si="15"/>
+        <v>25.928114550459426</v>
+      </c>
+      <c r="H11" s="6">
+        <f t="shared" si="3"/>
+        <v>0.69955072139860208</v>
+      </c>
+      <c r="I11" s="9">
+        <f t="shared" si="16"/>
+        <v>69.955072139860206</v>
+      </c>
+      <c r="J11" s="9">
         <f t="shared" si="11"/>
-        <v>74.071885449540574</v>
-      </c>
-      <c r="G11" s="9">
-        <f t="shared" si="12"/>
-        <v>25.928114550459426</v>
-      </c>
-      <c r="H11" s="6">
-        <f>(E11-N$10/100)/(1-N$10/100)</f>
-        <v>0.69955072139860208</v>
-      </c>
-      <c r="I11" s="9">
-        <f t="shared" si="13"/>
-        <v>69.955072139860206</v>
-      </c>
-      <c r="J11" s="9">
-        <f t="shared" si="8"/>
         <v>30.044927860139794</v>
       </c>
       <c r="K11" s="10">
-        <f>-1/($K$29+$K$28*G11)</f>
+        <f t="shared" si="4"/>
         <v>-3.508401961228484</v>
       </c>
       <c r="L11" s="10">
-        <f>A11-K11</f>
+        <f t="shared" si="5"/>
         <v>0.13840196122848392</v>
       </c>
       <c r="M11" s="81" t="s">
@@ -21229,39 +21229,39 @@
         <v>1.54162</v>
       </c>
       <c r="D12" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>9.2500000000000082E-2</v>
       </c>
       <c r="E12" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.66090955957196007</v>
       </c>
       <c r="F12" s="9">
+        <f t="shared" si="14"/>
+        <v>66.090955957196002</v>
+      </c>
+      <c r="G12" s="9">
+        <f t="shared" si="15"/>
+        <v>33.909044042803998</v>
+      </c>
+      <c r="H12" s="6">
+        <f t="shared" si="3"/>
+        <v>0.60706946890039215</v>
+      </c>
+      <c r="I12" s="9">
+        <f t="shared" si="16"/>
+        <v>60.706946890039212</v>
+      </c>
+      <c r="J12" s="9">
         <f t="shared" si="11"/>
-        <v>66.090955957196002</v>
-      </c>
-      <c r="G12" s="9">
-        <f t="shared" si="12"/>
-        <v>33.909044042803998</v>
-      </c>
-      <c r="H12" s="6">
-        <f>(E12-N$10/100)/(1-N$10/100)</f>
-        <v>0.60706946890039215</v>
-      </c>
-      <c r="I12" s="9">
-        <f t="shared" si="13"/>
-        <v>60.706946890039212</v>
-      </c>
-      <c r="J12" s="9">
-        <f t="shared" si="8"/>
         <v>39.293053109960788</v>
       </c>
       <c r="K12" s="10">
-        <f>-1/($K$29+$K$28*G12)</f>
+        <f t="shared" si="4"/>
         <v>-4.0428735897050334</v>
       </c>
       <c r="L12" s="10">
-        <f>A12-K12</f>
+        <f t="shared" si="5"/>
         <v>-0.22712641029496616</v>
       </c>
       <c r="M12" s="70" t="s">
@@ -21288,39 +21288,39 @@
         <v>1.52616</v>
       </c>
       <c r="D13" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>7.7040000000000053E-2</v>
       </c>
       <c r="E13" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.55044835102079781</v>
       </c>
       <c r="F13" s="9">
+        <f t="shared" si="14"/>
+        <v>55.04483510207978</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" si="15"/>
+        <v>44.95516489792022</v>
+      </c>
+      <c r="H13" s="6">
+        <f t="shared" si="3"/>
+        <v>0.47906945425201813</v>
+      </c>
+      <c r="I13" s="9">
+        <f t="shared" si="16"/>
+        <v>47.906945425201812</v>
+      </c>
+      <c r="J13" s="9">
         <f t="shared" si="11"/>
-        <v>55.04483510207978</v>
-      </c>
-      <c r="G13" s="9">
-        <f t="shared" si="12"/>
-        <v>44.95516489792022</v>
-      </c>
-      <c r="H13" s="6">
-        <f>(E13-N$10/100)/(1-N$10/100)</f>
-        <v>0.47906945425201813</v>
-      </c>
-      <c r="I13" s="9">
-        <f t="shared" si="13"/>
-        <v>47.906945425201812</v>
-      </c>
-      <c r="J13" s="9">
-        <f t="shared" si="8"/>
         <v>52.093054574798188</v>
       </c>
       <c r="K13" s="10">
-        <f>-1/($K$29+$K$28*G13)</f>
+        <f t="shared" si="4"/>
         <v>-5.1230674407443031</v>
       </c>
       <c r="L13" s="10">
-        <f>A13-K13</f>
+        <f t="shared" si="5"/>
         <v>-0.22893255925569722</v>
       </c>
       <c r="M13" s="72" t="s">
@@ -21347,39 +21347,39 @@
         <v>1.5079100000000001</v>
       </c>
       <c r="D14" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>5.8790000000000175E-2</v>
       </c>
       <c r="E14" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.42005268115930394</v>
       </c>
       <c r="F14" s="9">
+        <f t="shared" si="14"/>
+        <v>42.005268115930392</v>
+      </c>
+      <c r="G14" s="9">
+        <f t="shared" si="15"/>
+        <v>57.994731884069608</v>
+      </c>
+      <c r="H14" s="6">
+        <f t="shared" si="3"/>
+        <v>0.32796982505843414</v>
+      </c>
+      <c r="I14" s="9">
+        <f t="shared" si="16"/>
+        <v>32.796982505843417</v>
+      </c>
+      <c r="J14" s="9">
         <f t="shared" si="11"/>
-        <v>42.005268115930392</v>
-      </c>
-      <c r="G14" s="9">
-        <f t="shared" si="12"/>
-        <v>57.994731884069608</v>
-      </c>
-      <c r="H14" s="6">
-        <f>(E14-N$10/100)/(1-N$10/100)</f>
-        <v>0.32796982505843414</v>
-      </c>
-      <c r="I14" s="9">
-        <f t="shared" si="13"/>
-        <v>32.796982505843417</v>
-      </c>
-      <c r="J14" s="9">
-        <f t="shared" si="8"/>
         <v>67.203017494156583</v>
       </c>
       <c r="K14" s="10">
-        <f>-1/($K$29+$K$28*G14)</f>
+        <f t="shared" si="4"/>
         <v>-7.4833260117645723</v>
       </c>
       <c r="L14" s="10">
-        <f>A14-K14</f>
+        <f t="shared" si="5"/>
         <v>0.51132601176457193</v>
       </c>
       <c r="M14" s="74" t="s">
@@ -21544,19 +21544,19 @@
         <v>1.5953900000000001</v>
       </c>
       <c r="D20" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.14627000000000018</v>
       </c>
       <c r="E20" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>1.0450945003090879</v>
       </c>
       <c r="F20" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>104.50945003090879</v>
       </c>
       <c r="G20" s="9">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>-4.5094500309087948</v>
       </c>
       <c r="H20" s="6">
@@ -21564,15 +21564,15 @@
         <v>1.0522545133792458</v>
       </c>
       <c r="I20" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>105.22545133792458</v>
       </c>
       <c r="J20" s="10">
-        <f t="shared" ref="J20" si="14">-1/($K$29+$K$28*G20)</f>
+        <f t="shared" ref="J20" si="17">-1/($K$29+$K$28*G20)</f>
         <v>-2.3324253702194326</v>
       </c>
       <c r="K20" s="10">
-        <f t="shared" ref="K20" si="15">A20-J20</f>
+        <f t="shared" ref="K20" si="18">A20-J20</f>
         <v>2.0504253702194326</v>
       </c>
       <c r="M20" s="19"/>

</xml_diff>

<commit_message>
updated vignettes and function descriptions with links to the vignettes
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159EDE11-BF95-5D49-BFF6-A4914956087A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA70EF0-F1A6-EA40-83E4-A793FD549D94}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6669,7 +6669,7 @@
         <c:axId val="415423264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="0"/>
+          <c:min val="8.0000000000000016E-2"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -15538,16 +15538,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>498605</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>602278</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>121104</xdr:rowOff>
+      <xdr:rowOff>82227</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>608044</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>76717</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>149679</xdr:rowOff>
+      <xdr:rowOff>110802</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15615,15 +15615,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>1003041</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>164064</xdr:rowOff>
+      <xdr:colOff>3089470</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>60391</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>458755</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>123631</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>199572</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>149549</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15650,16 +15650,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>505406</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>148512</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>3174999</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>122594</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>2542590</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>92529</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>624631</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>66611</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15686,16 +15686,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>495687</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>3693</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>923341</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>16653</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>1500672</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>25464</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>321386</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>38424</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -18011,10 +18011,6 @@
         <f>-STDEV(B13:B16)/STDEV(G13:G16)</f>
         <v>-4.1640914464771868E-3</v>
       </c>
-      <c r="M22">
-        <f>0.003*21</f>
-        <v>6.3E-2</v>
-      </c>
     </row>
     <row r="23" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">

</xml_diff>

<commit_message>
its in a state with optim is implemented but not tested
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA70EF0-F1A6-EA40-83E4-A793FD549D94}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B6A7D8-6DFF-EA48-9108-824B7FB98E20}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15920" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="procedure" sheetId="18" r:id="rId1"/>

</xml_diff>

<commit_message>
clean test with new optim
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B6A7D8-6DFF-EA48-9108-824B7FB98E20}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B01EC5-FF03-CE4A-92D0-685442D5E373}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15920" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15920" tabRatio="578" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="procedure" sheetId="18" r:id="rId1"/>
@@ -2238,6 +2238,545 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Symbol"/>
+              </a:rPr>
+              <a:t>Y</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="-25000">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>TLP</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.47982076467245716"/>
+          <c:y val="6.5420560747663545E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="25400">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.12174971681702335"/>
+          <c:y val="0.1190842510415248"/>
+          <c:w val="0.8455039227519614"/>
+          <c:h val="0.68257491675915649"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>QUAG_3!$G$8:$G$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>4.2545509819495209</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.8036668538089771</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11.607602986213848</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15.343313244658475</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>19.434129040978092</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>QUAG_3!$B$8:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1.2547051442910915</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.51546391752577325</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.40551500405515001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.3427004797806717</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.26881720430107525</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-577B-4931-A592-C94E3C488AD4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="3175">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:forward val="1"/>
+            <c:backward val="5"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.28935185185185186"/>
+                  <c:y val="-0.36220122484689415"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="#,##0.000000" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln w="25400">
+                  <a:noFill/>
+                </a:ln>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                      <a:ea typeface="Calibri"/>
+                      <a:cs typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>QUAG_3!$G$12:$G$16</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>19.434129040978092</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>23.155635077907718</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>26.451014469387445</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>29.438635728042087</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>QUAG_3!$B$12:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.26881720430107525</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.26730820636193531</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.23854961832061067</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.18935807612194661</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-577B-4931-A592-C94E3C488AD4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="415417360"/>
+        <c:axId val="1"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="415417360"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="35"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                    <a:cs typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>100- total RWC (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.43049338420326327"/>
+              <c:y val="0.897199205239532"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="25400">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="3175">
+            <a:solidFill>
+              <a:srgbClr val="808080"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" vert="horz"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1.3"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                    <a:ea typeface="Calibri"/>
+                    <a:cs typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>1/</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Symbol"/>
+                  </a:rPr>
+                  <a:t>Y</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t> (MPa</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="30000">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>-1</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="2.985777138986976E-2"/>
+              <c:y val="0.23987651919449918"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="25400">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="3175">
+            <a:solidFill>
+              <a:srgbClr val="808080"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" vert="horz"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="415417360"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="25400">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="3175">
+      <a:solidFill>
+        <a:srgbClr val="808080"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:latin typeface="Calibri"/>
+          <a:ea typeface="Calibri"/>
+          <a:cs typeface="Calibri"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter alignWithMargins="0"/>
+    <c:pageMargins b="0.75000000000000289" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000289" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout>
@@ -2623,7 +3162,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3174,7 +3713,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3579,7 +4118,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3940,7 +4479,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4473,7 +5012,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4866,7 +5405,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -5372,7 +5911,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -5738,7 +6277,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -6051,368 +6590,6 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1084507279"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:intercept val="0"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>summary!$F$2:$F$6</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>70.776892607934158</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>62.483637277180918</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>84.656686755341525</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>75.609937703193737</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>74.071885449540574</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>summary!$R$2:$R$6</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>75.950675756694906</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>54.538844485554485</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>85.878197198208625</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>73.838702898533015</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>72.649175357052727</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-208C-4F29-BB4A-CABC3E5DB35E}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="982204079"/>
-        <c:axId val="982221135"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="982204079"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="982221135"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="982221135"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="982204079"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -6918,6 +7095,368 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>summary!$F$2:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>70.776892607934158</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>62.483637277180918</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>84.656686755341525</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>75.609937703193737</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>74.071885449540574</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>summary!$R$2:$R$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>75.950675756694906</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>54.538844485554485</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>85.878197198208625</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>73.838702898533015</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>72.649175357052727</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-208C-4F29-BB4A-CABC3E5DB35E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="982204079"/>
+        <c:axId val="982221135"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="982204079"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="982221135"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="982221135"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="982204079"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
       <c:layout>
         <c:manualLayout>
           <c:layoutTarget val="inner"/>
@@ -7244,7 +7783,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart22.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -8715,6 +9254,358 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>QUAG_1!$C$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>M(g)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>QUAG_1!$C$8:$C$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>1.69065</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.6804699999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.67065</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0.0000">
+                  <c:v>1.6553199999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.6475299999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.6378999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.6173500000000001</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.0000">
+                  <c:v>1.6086100000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.5931599999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>QUAG_1!$A$8:$A$16</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>-0.65200000000000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1.095</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.9650000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-2.6509999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-2.7919999999999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-2.8580000000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-3.2970000000000002</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-3.3079999999999998</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-3.9039999999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-78AC-2A4E-8F35-B0765AC27D33}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2007730992"/>
+        <c:axId val="2007732640"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2007730992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2007732640"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2007732640"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2007730992"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
       <c:tx>
         <c:rich>
           <a:bodyPr/>
@@ -9238,7 +10129,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -9636,7 +10527,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -9991,546 +10882,47 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Symbol"/>
-              </a:rPr>
-              <a:t>Y</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="-25000">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>TLP</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.47982076467245716"/>
-          <c:y val="6.5420560747663545E-2"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln w="25400">
-          <a:noFill/>
-        </a:ln>
-      </c:spPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.12174971681702335"/>
-          <c:y val="0.1190842510415248"/>
-          <c:w val="0.8455039227519614"/>
-          <c:h val="0.68257491675915649"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="3175">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="6"/>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-              </a:ln>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>QUAG_3!$G$8:$G$12</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>4.2545509819495209</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>9.8036668538089771</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>11.607602986213848</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>15.343313244658475</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>19.434129040978092</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>QUAG_3!$B$8:$B$12</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>1.2547051442910915</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.51546391752577325</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.40551500405515001</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.3427004797806717</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.26881720430107525</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-577B-4931-A592-C94E3C488AD4}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:ln w="28575">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="6"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-              </a:ln>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:forward val="1"/>
-            <c:backward val="5"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="0.28935185185185186"/>
-                  <c:y val="-0.36220122484689415"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="#,##0.000000" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln w="25400">
-                  <a:noFill/>
-                </a:ln>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                      <a:solidFill>
-                        <a:srgbClr val="000000"/>
-                      </a:solidFill>
-                      <a:latin typeface="Calibri"/>
-                      <a:ea typeface="Calibri"/>
-                      <a:cs typeface="Calibri"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>QUAG_3!$G$12:$G$16</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>19.434129040978092</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>23.155635077907718</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>26.451014469387445</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>29.438635728042087</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>QUAG_3!$B$12:$B$16</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>0.26881720430107525</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.26730820636193531</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.23854961832061067</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.18935807612194661</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-577B-4931-A592-C94E3C488AD4}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="415417360"/>
-        <c:axId val="1"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="415417360"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="35"/>
-          <c:min val="0"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                    <a:ea typeface="Calibri"/>
-                    <a:cs typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>100- total RWC (%)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.43049338420326327"/>
-              <c:y val="0.897199205239532"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="25400">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
-        <c:numFmt formatCode="0" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="out"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln w="3175">
-            <a:solidFill>
-              <a:srgbClr val="808080"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="0" vert="horz"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1.3"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                    <a:ea typeface="Calibri"/>
-                    <a:cs typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>1/</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Symbol"/>
-                  </a:rPr>
-                  <a:t>Y</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t> (MPa</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="30000">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>-1</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="2.985777138986976E-2"/>
-              <c:y val="0.23987651919449918"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="25400">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
-        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="out"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln w="3175">
-            <a:solidFill>
-              <a:srgbClr val="808080"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="0" vert="horz"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="415417360"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln w="25400">
-          <a:noFill/>
-        </a:ln>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln w="3175">
-      <a:solidFill>
-        <a:srgbClr val="808080"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:latin typeface="Calibri"/>
-          <a:ea typeface="Calibri"/>
-          <a:cs typeface="Calibri"/>
-        </a:defRPr>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter alignWithMargins="0"/>
-    <c:pageMargins b="0.75000000000000289" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000289" header="0.30000000000000032" footer="0.30000000000000032"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -11406,6 +11798,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -15715,6 +16623,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>701092</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>60390</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>918806</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>146957</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{792D5C46-49E6-8648-9415-DFA7590C55E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>

<commit_message>
working through nonlinear solutions
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819BB8F0-458B-7D4E-81FB-CD3FD9C44992}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1C7F717-FEF9-8044-9D4E-5BC049B7458E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="160" yWindow="660" windowWidth="15440" windowHeight="17180" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27660" windowHeight="17500" tabRatio="578" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="procedure" sheetId="18" r:id="rId1"/>
@@ -12473,36 +12473,36 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'QUAG_1 (2)'!$C$8:$C$16</c:f>
+              <c:f>'QUAG_1 (2)'!$N$8:$N$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1.69065</c:v>
+                  <c:v>-0.79982047331926309</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.6804699999999999</c:v>
+                  <c:v>-1.2874347622885982</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.67065</c:v>
-                </c:pt>
-                <c:pt idx="3" formatCode="0.0000">
-                  <c:v>1.6553199999999999</c:v>
+                  <c:v>-1.7439343393883371</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-2.411197253488754</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.6475299999999999</c:v>
+                  <c:v>-2.6944509347004142</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6378999999999999</c:v>
+                  <c:v>-2.8580000000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.6173500000000001</c:v>
-                </c:pt>
-                <c:pt idx="7" formatCode="0.0000">
-                  <c:v>1.6086100000000001</c:v>
+                  <c:v>-3.2970000000000002</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-3.3079999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5931599999999999</c:v>
+                  <c:v>-3.9039999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12582,7 +12582,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -23069,15 +23069,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>163286</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>66869</xdr:rowOff>
+      <xdr:colOff>901959</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>27992</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>614265</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>166396</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>458755</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -23104,16 +23104,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>707572</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>15033</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>357673</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>170543</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>82939</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>166396</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>886408</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>179355</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -23872,16 +23872,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>701092</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>60390</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>27215</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>138145</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>918806</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>146957</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>841052</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>159917</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -25933,11 +25933,11 @@
         <v>1.1846288130401266</v>
       </c>
       <c r="M9" s="10">
-        <f t="shared" ref="M9:M16" si="5">-H$12*P$9*((H9-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
+        <f>-H$12*P$9*((H9-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
         <v>0.99219405075152911</v>
       </c>
       <c r="N9" s="10">
-        <f t="shared" ref="N9:N16" si="6">K9+M9</f>
+        <f>K9+M9</f>
         <v>-1.2874347622885982</v>
       </c>
       <c r="O9" s="67" t="s">
@@ -25964,11 +25964,11 @@
         <v>1.67065</v>
       </c>
       <c r="D10" s="7">
-        <f t="shared" ref="D10:D16" si="7">C10-$B$3-$B$4</f>
+        <f t="shared" ref="D10:D16" si="5">C10-$B$3-$B$4</f>
         <v>0.16687000000000002</v>
       </c>
       <c r="E10" s="6">
-        <f t="shared" ref="E10:E16" si="8">(D10/$B$23)</f>
+        <f t="shared" ref="E10:E16" si="6">(D10/$B$23)</f>
         <v>0.8216027874425027</v>
       </c>
       <c r="F10" s="9">
@@ -25980,15 +25980,15 @@
         <v>17.839721255749737</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" ref="H10:H16" si="9">(E10-P$10/100)/(1-P$10/100)</f>
+        <f t="shared" ref="H10:H16" si="7">(E10-P$10/100)/(1-P$10/100)</f>
         <v>0.849263204905084</v>
       </c>
       <c r="I10" s="9">
-        <f t="shared" ref="I10:I16" si="10">H10*100</f>
+        <f t="shared" ref="I10:I16" si="8">H10*100</f>
         <v>84.926320490508402</v>
       </c>
       <c r="J10" s="10">
-        <f t="shared" ref="J10:J16" si="11">-1/($L$23+$L$22*G10)</f>
+        <f t="shared" ref="J10:J16" si="9">-1/($L$23+$L$22*G10)</f>
         <v>-2.3892887944870718</v>
       </c>
       <c r="K10" s="10">
@@ -26000,11 +26000,11 @@
         <v>0.42428879448707169</v>
       </c>
       <c r="M10" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="M9:M16" si="10">-H$12*P$9*((H10-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
         <v>0.64535445509873468</v>
       </c>
       <c r="N10" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="N10:N12" si="11">K10+M10</f>
         <v>-1.7439343393883371</v>
       </c>
       <c r="O10" s="62" t="s">
@@ -26031,11 +26031,11 @@
         <v>1.6553199999999999</v>
       </c>
       <c r="D11" s="26">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.15153999999999995</v>
       </c>
       <c r="E11" s="27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.74612384736044113</v>
       </c>
       <c r="F11" s="28">
@@ -26047,15 +26047,15 @@
         <v>25.387615263955894</v>
       </c>
       <c r="H11" s="27">
+        <f t="shared" si="7"/>
+        <v>0.78548724472036868</v>
+      </c>
+      <c r="I11" s="28">
+        <f t="shared" si="8"/>
+        <v>78.548724472036866</v>
+      </c>
+      <c r="J11" s="29">
         <f t="shared" si="9"/>
-        <v>0.78548724472036868</v>
-      </c>
-      <c r="I11" s="28">
-        <f t="shared" si="10"/>
-        <v>78.548724472036866</v>
-      </c>
-      <c r="J11" s="29">
-        <f t="shared" si="11"/>
         <v>-2.5832819981338613</v>
       </c>
       <c r="K11" s="10">
@@ -26067,11 +26067,11 @@
         <v>-6.7718001866138522E-2</v>
       </c>
       <c r="M11" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>0.17208474464510742</v>
       </c>
       <c r="N11" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v>-2.411197253488754</v>
       </c>
       <c r="O11" s="81" t="s">
@@ -26098,11 +26098,11 @@
         <v>1.6475299999999999</v>
       </c>
       <c r="D12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.14374999999999999</v>
       </c>
       <c r="E12" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.70776892607934161</v>
       </c>
       <c r="F12" s="9">
@@ -26114,19 +26114,19 @@
         <v>29.223107392065842</v>
       </c>
       <c r="H12" s="6">
+        <f t="shared" si="7"/>
+        <v>0.75307923886003403</v>
+      </c>
+      <c r="I12" s="9">
+        <f t="shared" si="8"/>
+        <v>75.307923886003408</v>
+      </c>
+      <c r="J12" s="10">
         <f t="shared" si="9"/>
-        <v>0.75307923886003403</v>
-      </c>
-      <c r="I12" s="9">
-        <f t="shared" si="10"/>
-        <v>75.307923886003408</v>
-      </c>
-      <c r="J12" s="10">
-        <f t="shared" si="11"/>
         <v>-2.6944509347004142</v>
       </c>
       <c r="K12" s="10">
-        <f t="shared" si="3"/>
+        <f>(P$9*H$12)/H12</f>
         <v>-2.6944509347004142</v>
       </c>
       <c r="L12" s="10">
@@ -26134,11 +26134,11 @@
         <v>-9.7549065299585624E-2</v>
       </c>
       <c r="M12" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N12" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v>-2.6944509347004142</v>
       </c>
       <c r="O12" s="70" t="s">
@@ -26165,11 +26165,11 @@
         <v>1.6378999999999999</v>
       </c>
       <c r="D13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.13411999999999996</v>
       </c>
       <c r="E13" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.66035456254442626</v>
       </c>
       <c r="F13" s="9">
@@ -26181,15 +26181,15 @@
         <v>33.964543745557378</v>
       </c>
       <c r="H13" s="6">
+        <f t="shared" si="7"/>
+        <v>0.71301645369507582</v>
+      </c>
+      <c r="I13" s="9">
+        <f t="shared" si="8"/>
+        <v>71.301645369507582</v>
+      </c>
+      <c r="J13" s="10">
         <f t="shared" si="9"/>
-        <v>0.71301645369507582</v>
-      </c>
-      <c r="I13" s="9">
-        <f t="shared" si="10"/>
-        <v>71.301645369507582</v>
-      </c>
-      <c r="J13" s="10">
-        <f t="shared" si="11"/>
         <v>-2.8458460510052443</v>
       </c>
       <c r="K13" s="10">
@@ -26201,12 +26201,12 @@
         <v>-1.2153948994755748E-2</v>
       </c>
       <c r="M13" s="10" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>#NUM!</v>
       </c>
-      <c r="N13" s="10" t="e">
-        <f t="shared" si="6"/>
-        <v>#NUM!</v>
+      <c r="N13" s="10">
+        <f>A13</f>
+        <v>-2.8580000000000001</v>
       </c>
       <c r="O13" s="87" t="s">
         <v>83</v>
@@ -26232,11 +26232,11 @@
         <v>1.6173500000000001</v>
       </c>
       <c r="D14" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.11357000000000012</v>
       </c>
       <c r="E14" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.55917437867708464</v>
       </c>
       <c r="F14" s="9">
@@ -26248,15 +26248,15 @@
         <v>44.082562132291535</v>
       </c>
       <c r="H14" s="6">
+        <f t="shared" si="7"/>
+        <v>0.62752421743963638</v>
+      </c>
+      <c r="I14" s="9">
+        <f t="shared" si="8"/>
+        <v>62.752421743963637</v>
+      </c>
+      <c r="J14" s="10">
         <f t="shared" si="9"/>
-        <v>0.62752421743963638</v>
-      </c>
-      <c r="I14" s="9">
-        <f t="shared" si="10"/>
-        <v>62.752421743963637</v>
-      </c>
-      <c r="J14" s="10">
-        <f t="shared" si="11"/>
         <v>-3.2335565746434067</v>
       </c>
       <c r="K14" s="10">
@@ -26268,12 +26268,12 @@
         <v>-6.3443425356593419E-2</v>
       </c>
       <c r="M14" s="10" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>#NUM!</v>
       </c>
-      <c r="N14" s="10" t="e">
-        <f t="shared" si="6"/>
-        <v>#NUM!</v>
+      <c r="N14" s="10">
+        <f t="shared" ref="N14:N16" si="12">A14</f>
+        <v>-3.2970000000000002</v>
       </c>
       <c r="O14" s="88" t="s">
         <v>1</v>
@@ -26298,11 +26298,11 @@
         <v>1.6086100000000001</v>
       </c>
       <c r="D15" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.10483000000000015</v>
       </c>
       <c r="E15" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.5161420279714608</v>
       </c>
       <c r="F15" s="9">
@@ -26314,15 +26314,15 @@
         <v>48.385797202853922</v>
       </c>
       <c r="H15" s="6">
+        <f t="shared" si="7"/>
+        <v>0.59116401574267563</v>
+      </c>
+      <c r="I15" s="9">
+        <f t="shared" si="8"/>
+        <v>59.116401574267563</v>
+      </c>
+      <c r="J15" s="10">
         <f t="shared" si="9"/>
-        <v>0.59116401574267563</v>
-      </c>
-      <c r="I15" s="9">
-        <f t="shared" si="10"/>
-        <v>59.116401574267563</v>
-      </c>
-      <c r="J15" s="10">
-        <f t="shared" si="11"/>
         <v>-3.4324400758742146</v>
       </c>
       <c r="K15" s="10">
@@ -26334,12 +26334,12 @@
         <v>0.12444007587421479</v>
       </c>
       <c r="M15" s="10" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>#NUM!</v>
       </c>
-      <c r="N15" s="10" t="e">
-        <f t="shared" si="6"/>
-        <v>#NUM!</v>
+      <c r="N15" s="10">
+        <f t="shared" si="12"/>
+        <v>-3.3079999999999998</v>
       </c>
       <c r="O15" s="76" t="s">
         <v>86</v>
@@ -26365,11 +26365,11 @@
         <v>1.5931599999999999</v>
       </c>
       <c r="D16" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>8.9379999999999959E-2</v>
       </c>
       <c r="E16" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.44007225469893241</v>
       </c>
       <c r="F16" s="9">
@@ -26381,15 +26381,15 @@
         <v>55.992774530106757</v>
       </c>
       <c r="H16" s="6">
+        <f t="shared" si="7"/>
+        <v>0.5268888308207017</v>
+      </c>
+      <c r="I16" s="9">
+        <f t="shared" si="8"/>
+        <v>52.68888308207017</v>
+      </c>
+      <c r="J16" s="10">
         <f t="shared" si="9"/>
-        <v>0.5268888308207017</v>
-      </c>
-      <c r="I16" s="9">
-        <f t="shared" si="10"/>
-        <v>52.68888308207017</v>
-      </c>
-      <c r="J16" s="10">
-        <f t="shared" si="11"/>
         <v>-3.8511635478953661</v>
       </c>
       <c r="K16" s="10">
@@ -26401,12 +26401,12 @@
         <v>-5.2836452104633835E-2</v>
       </c>
       <c r="M16" s="10" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>#NUM!</v>
       </c>
-      <c r="N16" s="10" t="e">
-        <f t="shared" si="6"/>
-        <v>#NUM!</v>
+      <c r="N16" s="10">
+        <f t="shared" si="12"/>
+        <v>-3.9039999999999999</v>
       </c>
       <c r="O16" s="70" t="s">
         <v>87</v>
@@ -26489,7 +26489,7 @@
         <v>1.7219100000000001</v>
       </c>
       <c r="D19" s="7">
-        <f t="shared" ref="D19" si="12">C19-$B$3-$B$4</f>
+        <f t="shared" ref="D19" si="13">C19-$B$3-$B$4</f>
         <v>0.2181300000000001</v>
       </c>
       <c r="E19" s="6">
@@ -26497,19 +26497,19 @@
         <v>1.0739870319699956</v>
       </c>
       <c r="F19" s="9">
-        <f t="shared" ref="F19" si="13">100*E19</f>
+        <f t="shared" ref="F19" si="14">100*E19</f>
         <v>107.39870319699956</v>
       </c>
       <c r="G19" s="9">
-        <f t="shared" ref="G19" si="14">100-F19</f>
+        <f t="shared" ref="G19" si="15">100-F19</f>
         <v>-7.3987031969995627</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" ref="H19" si="15">(E19-P$10/100)/(1-P$10/100)</f>
+        <f t="shared" ref="H19" si="16">(E19-P$10/100)/(1-P$10/100)</f>
         <v>1.0625153718371456</v>
       </c>
       <c r="I19" s="9">
-        <f t="shared" ref="I19" si="16">H19*100</f>
+        <f t="shared" ref="I19" si="17">H19*100</f>
         <v>106.25153718371456</v>
       </c>
       <c r="J19" s="10">
@@ -26518,7 +26518,7 @@
       </c>
       <c r="K19" s="10"/>
       <c r="L19" s="10">
-        <f t="shared" ref="L19" si="17">A19-J19</f>
+        <f t="shared" ref="L19" si="18">A19-J19</f>
         <v>1.6097465437525034</v>
       </c>
       <c r="M19" s="10"/>
@@ -26713,7 +26713,7 @@
     <col min="9" max="9" width="15.1640625" customWidth="1"/>
     <col min="10" max="10" width="11.6640625" customWidth="1"/>
     <col min="11" max="11" width="11.1640625" customWidth="1"/>
-    <col min="12" max="12" width="5.5" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="59.6640625" customWidth="1"/>
@@ -26874,6 +26874,10 @@
         <f>A8-J8</f>
         <v>1.5240923933685906</v>
       </c>
+      <c r="L8" s="10">
+        <f>J8+K8</f>
+        <v>-0.65200000000000014</v>
+      </c>
       <c r="M8" s="62" t="s">
         <v>52</v>
       </c>
@@ -26929,6 +26933,10 @@
         <f t="shared" ref="K9:K10" si="5">A9-J9</f>
         <v>1.1846288130401266</v>
       </c>
+      <c r="L9" s="10">
+        <f t="shared" ref="L9:L16" si="6">J9+K9</f>
+        <v>-1.095</v>
+      </c>
       <c r="M9" s="67" t="s">
         <v>47</v>
       </c>
@@ -26953,11 +26961,11 @@
         <v>1.67065</v>
       </c>
       <c r="D10" s="7">
-        <f t="shared" ref="D10" si="6">C10-$B$3-$B$4</f>
+        <f t="shared" ref="D10" si="7">C10-$B$3-$B$4</f>
         <v>0.16687000000000002</v>
       </c>
       <c r="E10" s="6">
-        <f t="shared" ref="E10" si="7">(D10/$B$23)</f>
+        <f t="shared" ref="E10" si="8">(D10/$B$23)</f>
         <v>0.8216027874425027</v>
       </c>
       <c r="F10" s="9">
@@ -26969,20 +26977,24 @@
         <v>17.839721255749737</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" ref="H10" si="8">(E10-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" ref="H10" si="9">(E10-N$10/100)/(1-N$10/100)</f>
         <v>0.849263204905084</v>
       </c>
       <c r="I10" s="9">
-        <f t="shared" ref="I10" si="9">H10*100</f>
+        <f t="shared" ref="I10" si="10">H10*100</f>
         <v>84.926320490508402</v>
       </c>
       <c r="J10" s="10">
-        <f t="shared" ref="J10" si="10">-1/($K$23+$K$22*G10)</f>
+        <f t="shared" ref="J10" si="11">-1/($K$23+$K$22*G10)</f>
         <v>-2.3892887944870718</v>
       </c>
       <c r="K10" s="10">
         <f t="shared" si="5"/>
         <v>0.42428879448707169</v>
+      </c>
+      <c r="L10" s="10">
+        <f t="shared" si="6"/>
+        <v>-1.9650000000000001</v>
       </c>
       <c r="M10" s="62" t="s">
         <v>82</v>
@@ -27008,36 +27020,40 @@
         <v>1.6553199999999999</v>
       </c>
       <c r="D11" s="26">
-        <f t="shared" ref="D11:D16" si="11">C11-$B$3-$B$4</f>
+        <f t="shared" ref="D11:D16" si="12">C11-$B$3-$B$4</f>
         <v>0.15153999999999995</v>
       </c>
       <c r="E11" s="27">
-        <f t="shared" ref="E11:E16" si="12">(D11/$B$23)</f>
+        <f t="shared" ref="E11:E16" si="13">(D11/$B$23)</f>
         <v>0.74612384736044113</v>
       </c>
       <c r="F11" s="28">
-        <f t="shared" ref="F11:F16" si="13">100*E11</f>
+        <f t="shared" ref="F11:F16" si="14">100*E11</f>
         <v>74.612384736044106</v>
       </c>
       <c r="G11" s="28">
-        <f t="shared" ref="G11:G16" si="14">100-F11</f>
+        <f t="shared" ref="G11:G16" si="15">100-F11</f>
         <v>25.387615263955894</v>
       </c>
       <c r="H11" s="27">
-        <f t="shared" ref="H11:H16" si="15">(E11-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" ref="H11:H16" si="16">(E11-N$10/100)/(1-N$10/100)</f>
         <v>0.78548724472036868</v>
       </c>
       <c r="I11" s="28">
-        <f t="shared" ref="I11:I16" si="16">H11*100</f>
+        <f t="shared" ref="I11:I16" si="17">H11*100</f>
         <v>78.548724472036866</v>
       </c>
       <c r="J11" s="29">
-        <f t="shared" ref="J11:J16" si="17">-1/($K$23+$K$22*G11)</f>
+        <f t="shared" ref="J11:J16" si="18">-1/($K$23+$K$22*G11)</f>
         <v>-2.5832819981338613</v>
       </c>
       <c r="K11" s="29">
-        <f t="shared" ref="K11:K16" si="18">A11-J11</f>
+        <f t="shared" ref="K11:K16" si="19">A11-J11</f>
         <v>-6.7718001866138522E-2</v>
+      </c>
+      <c r="L11" s="10">
+        <f t="shared" si="6"/>
+        <v>-2.6509999999999998</v>
       </c>
       <c r="M11" s="81" t="s">
         <v>84</v>
@@ -27063,36 +27079,40 @@
         <v>1.6475299999999999</v>
       </c>
       <c r="D12" s="7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.14374999999999999</v>
       </c>
       <c r="E12" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.70776892607934161</v>
       </c>
       <c r="F12" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>70.776892607934158</v>
       </c>
       <c r="G12" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>29.223107392065842</v>
       </c>
       <c r="H12" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.75307923886003403</v>
       </c>
       <c r="I12" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>75.307923886003408</v>
       </c>
       <c r="J12" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-2.6944509347004142</v>
       </c>
       <c r="K12" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-9.7549065299585624E-2</v>
+      </c>
+      <c r="L12" s="10">
+        <f t="shared" si="6"/>
+        <v>-2.7919999999999998</v>
       </c>
       <c r="M12" s="70" t="s">
         <v>85</v>
@@ -27118,38 +27138,41 @@
         <v>1.6378999999999999</v>
       </c>
       <c r="D13" s="7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.13411999999999996</v>
       </c>
       <c r="E13" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.66035456254442626</v>
       </c>
       <c r="F13" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>66.035456254442622</v>
       </c>
       <c r="G13" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>33.964543745557378</v>
       </c>
       <c r="H13" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.71301645369507582</v>
       </c>
       <c r="I13" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>71.301645369507582</v>
       </c>
       <c r="J13" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-2.8458460510052443</v>
       </c>
       <c r="K13" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-1.2153948994755748E-2</v>
       </c>
-      <c r="L13" s="3"/>
+      <c r="L13" s="10">
+        <f t="shared" si="6"/>
+        <v>-2.8580000000000001</v>
+      </c>
       <c r="M13" s="87" t="s">
         <v>83</v>
       </c>
@@ -27174,38 +27197,41 @@
         <v>1.6173500000000001</v>
       </c>
       <c r="D14" s="7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.11357000000000012</v>
       </c>
       <c r="E14" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.55917437867708464</v>
       </c>
       <c r="F14" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>55.917437867708465</v>
       </c>
       <c r="G14" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>44.082562132291535</v>
       </c>
       <c r="H14" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.62752421743963638</v>
       </c>
       <c r="I14" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>62.752421743963637</v>
       </c>
       <c r="J14" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-3.2335565746434067</v>
       </c>
       <c r="K14" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-6.3443425356593419E-2</v>
       </c>
-      <c r="L14" s="3"/>
+      <c r="L14" s="10">
+        <f t="shared" si="6"/>
+        <v>-3.2970000000000002</v>
+      </c>
       <c r="M14" s="88" t="s">
         <v>1</v>
       </c>
@@ -27229,36 +27255,40 @@
         <v>1.6086100000000001</v>
       </c>
       <c r="D15" s="7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.10483000000000015</v>
       </c>
       <c r="E15" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.5161420279714608</v>
       </c>
       <c r="F15" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>51.614202797146078</v>
       </c>
       <c r="G15" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>48.385797202853922</v>
       </c>
       <c r="H15" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.59116401574267563</v>
       </c>
       <c r="I15" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>59.116401574267563</v>
       </c>
       <c r="J15" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-3.4324400758742146</v>
       </c>
       <c r="K15" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.12444007587421479</v>
+      </c>
+      <c r="L15" s="10">
+        <f t="shared" si="6"/>
+        <v>-3.3079999999999998</v>
       </c>
       <c r="M15" s="76" t="s">
         <v>86</v>
@@ -27284,36 +27314,40 @@
         <v>1.5931599999999999</v>
       </c>
       <c r="D16" s="7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>8.9379999999999959E-2</v>
       </c>
       <c r="E16" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.44007225469893241</v>
       </c>
       <c r="F16" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>44.007225469893243</v>
       </c>
       <c r="G16" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>55.992774530106757</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.5268888308207017</v>
       </c>
       <c r="I16" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>52.68888308207017</v>
       </c>
       <c r="J16" s="10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-3.8511635478953661</v>
       </c>
       <c r="K16" s="10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-5.2836452104633835E-2</v>
+      </c>
+      <c r="L16" s="10">
+        <f t="shared" si="6"/>
+        <v>-3.9039999999999999</v>
       </c>
       <c r="M16" s="70" t="s">
         <v>87</v>
@@ -27392,7 +27426,7 @@
         <v>1.7219100000000001</v>
       </c>
       <c r="D19" s="7">
-        <f t="shared" ref="D19" si="19">C19-$B$3-$B$4</f>
+        <f t="shared" ref="D19" si="20">C19-$B$3-$B$4</f>
         <v>0.2181300000000001</v>
       </c>
       <c r="E19" s="6">
@@ -27400,19 +27434,19 @@
         <v>1.0739870319699956</v>
       </c>
       <c r="F19" s="9">
-        <f t="shared" ref="F19" si="20">100*E19</f>
+        <f t="shared" ref="F19" si="21">100*E19</f>
         <v>107.39870319699956</v>
       </c>
       <c r="G19" s="9">
-        <f t="shared" ref="G19" si="21">100-F19</f>
+        <f t="shared" ref="G19" si="22">100-F19</f>
         <v>-7.3987031969995627</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" ref="H19" si="22">(E19-N$10/100)/(1-N$10/100)</f>
+        <f t="shared" ref="H19" si="23">(E19-N$10/100)/(1-N$10/100)</f>
         <v>1.0625153718371456</v>
       </c>
       <c r="I19" s="9">
-        <f t="shared" ref="I19" si="23">H19*100</f>
+        <f t="shared" ref="I19" si="24">H19*100</f>
         <v>106.25153718371456</v>
       </c>
       <c r="J19" s="10">
@@ -27420,7 +27454,7 @@
         <v>-1.9097465437525034</v>
       </c>
       <c r="K19" s="10">
-        <f t="shared" ref="K19" si="24">A19-J19</f>
+        <f t="shared" ref="K19" si="25">A19-J19</f>
         <v>1.6097465437525034</v>
       </c>
       <c r="M19" s="60" t="s">

</xml_diff>

<commit_message>
put the nonlinear psip in osmest
</commit_message>
<xml_diff>
--- a/inst/extdata/QUAGaf_LS.xlsx
+++ b/inst/extdata/QUAGaf_LS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mr.bean/Documents/Research_UCLA/Packages/pvest/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1C7F717-FEF9-8044-9D4E-5BC049B7458E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F1E45C-970F-AA43-B18F-6DBE96A31696}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="27660" windowHeight="17500" tabRatio="578" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27660" windowHeight="17500" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="procedure" sheetId="18" r:id="rId1"/>
@@ -11799,16 +11799,16 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.5240923933685906</c:v>
+                  <c:v>1.6002356121316574</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1846288130401266</c:v>
+                  <c:v>1.2579576322767168</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.42428879448707169</c:v>
+                  <c:v>0.49403915887376848</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-6.7718001866138522E-2</c:v>
+                  <c:v>-5.7877793378704467E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12174,19 +12174,19 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1.5240923933685906</c:v>
+                  <c:v>1.6002356121316574</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1846288130401266</c:v>
+                  <c:v>1.2579576322767168</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.42428879448707169</c:v>
+                  <c:v>0.49403915887376848</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-6.7718001866138522E-2</c:v>
+                  <c:v>-5.7877793378704467E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-9.7549065299585624E-2</c:v>
+                  <c:v>-4.0948868588155829E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12478,19 +12478,19 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-0.79982047331926309</c:v>
+                  <c:v>-0.80684889273490246</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1.2874347622885982</c:v>
+                  <c:v>-1.3014833426440615</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1.7439343393883371</c:v>
+                  <c:v>-1.7669595383257493</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2.411197253488754</c:v>
+                  <c:v>-2.4538111788250165</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2.6944509347004142</c:v>
+                  <c:v>-2.7510511314118444</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>-2.8580000000000001</c:v>
@@ -12843,19 +12843,19 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-0.79982047331926309</c:v>
+                  <c:v>-0.80684889273490246</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1.2874347622885982</c:v>
+                  <c:v>-1.3014833426440615</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1.7439343393883371</c:v>
+                  <c:v>-1.7669595383257493</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2.411197253488754</c:v>
+                  <c:v>-2.4538111788250165</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2.6944509347004142</c:v>
+                  <c:v>-2.7510511314118444</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13136,31 +13136,31 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-2.1760923933685912</c:v>
+                  <c:v>-2.252235612131658</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-2.2796288130401274</c:v>
+                  <c:v>-2.3529576322767172</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-2.3892887944870718</c:v>
+                  <c:v>-2.459039158873769</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2.5832819981338613</c:v>
+                  <c:v>-2.6452122206621298</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2.6944509347004142</c:v>
+                  <c:v>-2.7510511314118444</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-2.8458460510052443</c:v>
+                  <c:v>-2.8942049553420248</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-3.2335565746434072</c:v>
+                  <c:v>-3.2557298343410244</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-3.4324400758742151</c:v>
+                  <c:v>-3.4383987955683208</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-3.851163547895367</c:v>
+                  <c:v>-3.8169744713674598</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13172,31 +13172,31 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1.5240923933685906</c:v>
+                  <c:v>1.6002356121316574</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1846288130401266</c:v>
+                  <c:v>1.2579576322767168</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.42428879448707169</c:v>
+                  <c:v>0.49403915887376848</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-6.7718001866138522E-2</c:v>
+                  <c:v>-5.7877793378704467E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-9.7549065299585624E-2</c:v>
+                  <c:v>-4.0948868588155829E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-1.2153948994755748E-2</c:v>
+                  <c:v>3.6204955342023837E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-6.3443425356593419E-2</c:v>
+                  <c:v>-4.1270165658976676E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.12444007587421479</c:v>
+                  <c:v>0.13039879556832012</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-5.2836452104633835E-2</c:v>
+                  <c:v>-8.7025528632540983E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -23068,16 +23068,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>901959</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>565020</xdr:colOff>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>27992</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>458755</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>393959</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>49763</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -25847,38 +25847,38 @@
       </c>
       <c r="H8" s="6">
         <f>(E8-P$10/100)/(1-P$10/100)</f>
-        <v>0.93246732778142483</v>
+        <v>0.93610233960373568</v>
       </c>
       <c r="I8" s="9">
         <f>H8*100</f>
-        <v>93.246732778142487</v>
+        <v>93.610233960373563</v>
       </c>
       <c r="J8" s="10">
         <f>-1/($L$23+$L$22*G8)</f>
-        <v>-2.1760923933685907</v>
+        <v>-2.2522356121316576</v>
       </c>
       <c r="K8" s="10">
         <f>(P$9*H$12)/H8</f>
-        <v>-2.1760923933685912</v>
+        <v>-2.252235612131658</v>
       </c>
       <c r="L8" s="10">
         <f>A8-J8</f>
-        <v>1.5240923933685906</v>
+        <v>1.6002356121316574</v>
       </c>
       <c r="M8" s="10">
         <f>-H$12*P$9*((H8-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
-        <v>1.3762719200493281</v>
+        <v>1.4453867193967556</v>
       </c>
       <c r="N8" s="10">
         <f>K8+M8</f>
-        <v>-0.79982047331926309</v>
+        <v>-0.80684889273490246</v>
       </c>
       <c r="O8" s="62" t="s">
         <v>52</v>
       </c>
       <c r="P8" s="66">
         <f>-1/L23</f>
-        <v>-2.0291350590498949</v>
+        <v>-2.1083230258552965</v>
       </c>
       <c r="Q8" t="s">
         <v>8</v>
@@ -25914,38 +25914,38 @@
       </c>
       <c r="H9" s="6">
         <f>(E9-P$10/100)/(1-P$10/100)</f>
-        <v>0.890116429237367</v>
+        <v>0.89603101940058638</v>
       </c>
       <c r="I9" s="9">
         <f>H9*100</f>
-        <v>89.011642923736702</v>
+        <v>89.603101940058636</v>
       </c>
       <c r="J9" s="10">
         <f>-1/($L$23+$L$22*G9)</f>
-        <v>-2.2796288130401265</v>
+        <v>-2.3529576322767167</v>
       </c>
       <c r="K9" s="10">
         <f t="shared" ref="K9:K16" si="3">(P$9*H$12)/H9</f>
-        <v>-2.2796288130401274</v>
+        <v>-2.3529576322767172</v>
       </c>
       <c r="L9" s="10">
         <f t="shared" ref="L9:L16" si="4">A9-J9</f>
-        <v>1.1846288130401266</v>
+        <v>1.2579576322767168</v>
       </c>
       <c r="M9" s="10">
         <f>-H$12*P$9*((H9-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
-        <v>0.99219405075152911</v>
+        <v>1.0514742896326557</v>
       </c>
       <c r="N9" s="10">
         <f>K9+M9</f>
-        <v>-1.2874347622885982</v>
+        <v>-1.3014833426440615</v>
       </c>
       <c r="O9" s="67" t="s">
         <v>47</v>
       </c>
       <c r="P9" s="68">
         <f>J12</f>
-        <v>-2.6944509347004142</v>
+        <v>-2.751051131411844</v>
       </c>
       <c r="Q9" t="s">
         <v>67</v>
@@ -25981,38 +25981,38 @@
       </c>
       <c r="H10" s="6">
         <f t="shared" ref="H10:H16" si="7">(E10-P$10/100)/(1-P$10/100)</f>
-        <v>0.849263204905084</v>
+        <v>0.85737675963684179</v>
       </c>
       <c r="I10" s="9">
         <f t="shared" ref="I10:I16" si="8">H10*100</f>
-        <v>84.926320490508402</v>
+        <v>85.737675963684183</v>
       </c>
       <c r="J10" s="10">
         <f t="shared" ref="J10:J16" si="9">-1/($L$23+$L$22*G10)</f>
-        <v>-2.3892887944870718</v>
+        <v>-2.4590391588737686</v>
       </c>
       <c r="K10" s="10">
         <f t="shared" si="3"/>
-        <v>-2.3892887944870718</v>
+        <v>-2.459039158873769</v>
       </c>
       <c r="L10" s="10">
         <f t="shared" si="4"/>
-        <v>0.42428879448707169</v>
+        <v>0.49403915887376848</v>
       </c>
       <c r="M10" s="10">
-        <f t="shared" ref="M9:M16" si="10">-H$12*P$9*((H10-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
-        <v>0.64535445509873468</v>
+        <f t="shared" ref="M10:M16" si="10">-H$12*P$9*((H10-H$12)/(1-H$12))^((P$14*(1-H$12))/(-H$12*P$9))</f>
+        <v>0.69207962054801975</v>
       </c>
       <c r="N10" s="10">
         <f t="shared" ref="N10:N12" si="11">K10+M10</f>
-        <v>-1.7439343393883371</v>
+        <v>-1.7669595383257493</v>
       </c>
       <c r="O10" s="62" t="s">
         <v>82</v>
       </c>
       <c r="P10" s="63">
         <f>100+(L23/L22)</f>
-        <v>-18.350143006001986</v>
+        <v>-25.082849122799786</v>
       </c>
       <c r="Q10" t="s">
         <v>8</v>
@@ -26048,31 +26048,31 @@
       </c>
       <c r="H11" s="27">
         <f t="shared" si="7"/>
-        <v>0.78548724472036868</v>
+        <v>0.79703360259221745</v>
       </c>
       <c r="I11" s="28">
         <f t="shared" si="8"/>
-        <v>78.548724472036866</v>
+        <v>79.703360259221739</v>
       </c>
       <c r="J11" s="29">
         <f t="shared" si="9"/>
-        <v>-2.5832819981338613</v>
+        <v>-2.6452122206621294</v>
       </c>
       <c r="K11" s="10">
         <f t="shared" si="3"/>
-        <v>-2.5832819981338613</v>
+        <v>-2.6452122206621298</v>
       </c>
       <c r="L11" s="29">
         <f t="shared" si="4"/>
-        <v>-6.7718001866138522E-2</v>
+        <v>-5.7877793378704467E-3</v>
       </c>
       <c r="M11" s="10">
         <f t="shared" si="10"/>
-        <v>0.17208474464510742</v>
+        <v>0.19140104183711332</v>
       </c>
       <c r="N11" s="10">
         <f t="shared" si="11"/>
-        <v>-2.411197253488754</v>
+        <v>-2.4538111788250165</v>
       </c>
       <c r="O11" s="81" t="s">
         <v>84</v>
@@ -26115,23 +26115,23 @@
       </c>
       <c r="H12" s="6">
         <f t="shared" si="7"/>
-        <v>0.75307923886003403</v>
+        <v>0.76636998919511246</v>
       </c>
       <c r="I12" s="9">
         <f t="shared" si="8"/>
-        <v>75.307923886003408</v>
+        <v>76.636998919511242</v>
       </c>
       <c r="J12" s="10">
-        <f t="shared" si="9"/>
-        <v>-2.6944509347004142</v>
+        <f>-1/($L$23+$L$22*G12)</f>
+        <v>-2.751051131411844</v>
       </c>
       <c r="K12" s="10">
-        <f>(P$9*H$12)/H12</f>
-        <v>-2.6944509347004142</v>
+        <f t="shared" si="3"/>
+        <v>-2.7510511314118444</v>
       </c>
       <c r="L12" s="10">
         <f t="shared" si="4"/>
-        <v>-9.7549065299585624E-2</v>
+        <v>-4.0948868588155829E-2</v>
       </c>
       <c r="M12" s="10">
         <f t="shared" si="10"/>
@@ -26139,14 +26139,14 @@
       </c>
       <c r="N12" s="10">
         <f t="shared" si="11"/>
-        <v>-2.6944509347004142</v>
+        <v>-2.7510511314118444</v>
       </c>
       <c r="O12" s="70" t="s">
         <v>85</v>
       </c>
       <c r="P12" s="71">
         <f>I12</f>
-        <v>75.307923886003408</v>
+        <v>76.636998919511242</v>
       </c>
       <c r="Q12" t="s">
         <v>66</v>
@@ -26182,23 +26182,23 @@
       </c>
       <c r="H13" s="6">
         <f t="shared" si="7"/>
-        <v>0.71301645369507582</v>
+        <v>0.72846362244105289</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" si="8"/>
-        <v>71.301645369507582</v>
+        <v>72.846362244105293</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="9"/>
-        <v>-2.8458460510052443</v>
+        <v>-2.8942049553420239</v>
       </c>
       <c r="K13" s="10">
         <f t="shared" si="3"/>
-        <v>-2.8458460510052443</v>
+        <v>-2.8942049553420248</v>
       </c>
       <c r="L13" s="10">
         <f t="shared" si="4"/>
-        <v>-1.2153948994755748E-2</v>
+        <v>3.6204955342023837E-2</v>
       </c>
       <c r="M13" s="10" t="e">
         <f t="shared" si="10"/>
@@ -26213,7 +26213,7 @@
       </c>
       <c r="P13" s="73">
         <f>STDEV(L8:L12)/STDEV(E8:E12)</f>
-        <v>8.4368937702080515</v>
+        <v>8.5241983512899484</v>
       </c>
       <c r="Q13" t="s">
         <v>58</v>
@@ -26249,23 +26249,23 @@
       </c>
       <c r="H14" s="6">
         <f t="shared" si="7"/>
-        <v>0.62752421743963638</v>
+        <v>0.64757308902507016</v>
       </c>
       <c r="I14" s="9">
         <f t="shared" si="8"/>
-        <v>62.752421743963637</v>
+        <v>64.75730890250702</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="9"/>
-        <v>-3.2335565746434067</v>
+        <v>-3.2557298343410235</v>
       </c>
       <c r="K14" s="10">
         <f t="shared" si="3"/>
-        <v>-3.2335565746434072</v>
+        <v>-3.2557298343410244</v>
       </c>
       <c r="L14" s="10">
         <f t="shared" si="4"/>
-        <v>-6.3443425356593419E-2</v>
+        <v>-4.1270165658976676E-2</v>
       </c>
       <c r="M14" s="10" t="e">
         <f t="shared" si="10"/>
@@ -26280,7 +26280,7 @@
       </c>
       <c r="P14" s="75">
         <f>STDEV(L8:L12)/STDEV(H8:H12)</f>
-        <v>9.9850758423057062</v>
+        <v>10.662310162672195</v>
       </c>
       <c r="Q14" t="s">
         <v>65</v>
@@ -26315,23 +26315,23 @@
       </c>
       <c r="H15" s="6">
         <f t="shared" si="7"/>
-        <v>0.59116401574267563</v>
+        <v>0.61317001057953768</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" si="8"/>
-        <v>59.116401574267563</v>
+        <v>61.317001057953767</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="9"/>
-        <v>-3.4324400758742146</v>
+        <v>-3.43839879556832</v>
       </c>
       <c r="K15" s="10">
         <f t="shared" si="3"/>
-        <v>-3.4324400758742151</v>
+        <v>-3.4383987955683208</v>
       </c>
       <c r="L15" s="10">
         <f t="shared" si="4"/>
-        <v>0.12444007587421479</v>
+        <v>0.13039879556832012</v>
       </c>
       <c r="M15" s="10" t="e">
         <f t="shared" si="10"/>
@@ -26382,23 +26382,23 @@
       </c>
       <c r="H16" s="6">
         <f t="shared" si="7"/>
-        <v>0.5268888308207017</v>
+        <v>0.55235450005511155</v>
       </c>
       <c r="I16" s="9">
         <f t="shared" si="8"/>
-        <v>52.68888308207017</v>
+        <v>55.235450005511154</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="9"/>
-        <v>-3.8511635478953661</v>
+        <v>-3.8169744713674589</v>
       </c>
       <c r="K16" s="10">
         <f t="shared" si="3"/>
-        <v>-3.851163547895367</v>
+        <v>-3.8169744713674598</v>
       </c>
       <c r="L16" s="10">
         <f t="shared" si="4"/>
-        <v>-5.2836452104633835E-2</v>
+        <v>-8.7025528632540983E-2</v>
       </c>
       <c r="M16" s="10" t="e">
         <f t="shared" si="10"/>
@@ -26444,7 +26444,7 @@
       </c>
       <c r="P17" s="78">
         <f>STDEV(H8:H12)/STDEV(A8:A12)</f>
-        <v>7.8146893846319426E-2</v>
+        <v>7.394056121240794E-2</v>
       </c>
       <c r="Q17" t="s">
         <v>62</v>
@@ -26471,7 +26471,7 @@
       </c>
       <c r="P18" s="80">
         <f>STDEV(H12:H16)/STDEV(A12:A16)</f>
-        <v>0.20504101470884589</v>
+        <v>0.19400448249355007</v>
       </c>
       <c r="Q18" t="s">
         <v>63</v>
@@ -26506,20 +26506,20 @@
       </c>
       <c r="H19" s="6">
         <f t="shared" ref="H19" si="16">(E19-P$10/100)/(1-P$10/100)</f>
-        <v>1.0625153718371456</v>
+        <v>1.0591504210919909</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" ref="I19" si="17">H19*100</f>
-        <v>106.25153718371456</v>
+        <v>105.91504210919909</v>
       </c>
       <c r="J19" s="10">
         <f>-1/($L$23+$L$22*G19)</f>
-        <v>-1.9097465437525034</v>
+        <v>-1.9905794152275387</v>
       </c>
       <c r="K19" s="10"/>
       <c r="L19" s="10">
         <f t="shared" ref="L19" si="18">A19-J19</f>
-        <v>1.6097465437525034</v>
+        <v>1.6905794152275386</v>
       </c>
       <c r="M19" s="10"/>
       <c r="O19" s="60" t="s">
@@ -26584,8 +26584,8 @@
       </c>
       <c r="K22" s="49"/>
       <c r="L22" s="41">
-        <f>-STDEV(B13:B16)/STDEV(G13:G16)</f>
-        <v>-4.1640914464771868E-3</v>
+        <f>-STDEV(B11:B16)/STDEV(G11:G16)</f>
+        <v>-3.7919716618975436E-3</v>
       </c>
       <c r="M22" s="41"/>
     </row>
@@ -26605,8 +26605,8 @@
       </c>
       <c r="K23" s="49"/>
       <c r="L23" s="42">
-        <f>AVERAGE(B13:B16)-L22*AVERAGE(G13:G16)</f>
-        <v>0.49282081818064472</v>
+        <f>AVERAGE(B11:B16)-L22*AVERAGE(G11:G16)</f>
+        <v>0.47431061926306278</v>
       </c>
       <c r="M23" s="42"/>
       <c r="N23" s="31"/>
@@ -26629,7 +26629,7 @@
       <c r="K26" s="103"/>
       <c r="L26" s="103">
         <f>-1/L23</f>
-        <v>-2.0291350590498949</v>
+        <v>-2.1083230258552965</v>
       </c>
       <c r="M26" s="103"/>
       <c r="U26" s="16"/>
@@ -26642,7 +26642,7 @@
       <c r="K27" s="103"/>
       <c r="L27" s="103">
         <f>-L26</f>
-        <v>2.0291350590498949</v>
+        <v>2.1083230258552965</v>
       </c>
       <c r="M27" s="103"/>
     </row>
@@ -26653,7 +26653,7 @@
       <c r="K28" s="103"/>
       <c r="L28" s="103">
         <f>-(INTERCEPT(L8:L11,G8:G11)/(SLOPE(L8:L11,G8:G11)))</f>
-        <v>24.049324243305094</v>
+        <v>24.708205665833965</v>
       </c>
       <c r="M28" s="103"/>
     </row>
@@ -26664,7 +26664,7 @@
       <c r="K29" s="103"/>
       <c r="L29" s="103">
         <f>100-L28</f>
-        <v>75.950675756694906</v>
+        <v>75.291794334166042</v>
       </c>
       <c r="M29" s="103"/>
     </row>
@@ -26675,7 +26675,7 @@
       <c r="K30" s="103"/>
       <c r="L30" s="103">
         <f>-1/(L22*(L28)+L23)</f>
-        <v>-2.5466207777195269</v>
+        <v>-2.627307473906463</v>
       </c>
       <c r="M30" s="103"/>
     </row>
@@ -26686,7 +26686,7 @@
       <c r="K31" s="103"/>
       <c r="L31" s="103">
         <f>L27/((100-L29)/100)</f>
-        <v>8.4373890863680732</v>
+        <v>8.5328860151534442</v>
       </c>
       <c r="M31" s="103"/>
     </row>

</xml_diff>